<commit_message>
add table discret inputs generating
</commit_message>
<xml_diff>
--- a/templates/analog.xlsx
+++ b/templates/analog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d.sharygin\Desktop\Protocols\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D33CA784-C2A8-4631-B52E-E1FDE10B768D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C2F4813-D63A-4B9B-9B9A-8EFE1C40CB72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
   <si>
     <t>Измерительный канал</t>
   </si>
@@ -40,18 +40,12 @@
     <t>Фаза, °</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
     <t>Название таблицы</t>
   </si>
   <si>
     <t>Тэг</t>
   </si>
   <si>
-    <t>analog</t>
-  </si>
-  <si>
     <t>Величина, А(В)</t>
   </si>
   <si>
@@ -64,7 +58,10 @@
     <t>Максимальная погрешность, %</t>
   </si>
   <si>
-    <t>Проверка аналоговых каналов</t>
+    <t>Проверка аналоговых каналов (A{{N}})</t>
+  </si>
+  <si>
+    <t>analog{{N}}</t>
   </si>
 </sst>
 </file>
@@ -410,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.140625" bestFit="1" customWidth="1"/>
@@ -435,269 +432,29 @@
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G1" s="2"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -718,21 +475,22 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>